<commit_message>
All figures and data for real time PCR
</commit_message>
<xml_diff>
--- a/datasets/Second Real-Time All Paula mutants.xlsx
+++ b/datasets/Second Real-Time All Paula mutants.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wageningenur4-my.sharepoint.com/personal/luciana_chavezrodriguez_wur_nl/Documents/UCI_projects/Project_8 (Reviews)/Family/Pere/doctorado/datasets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucia\OneDrive - Wageningen University &amp; Research\UCI_projects\Project_8 (Reviews)\Family\Pere\doctorado\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="92" documentId="11_F259E0D325B1EFF6C33EB1C278D77CAF535ECB94" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97C8D6F3-C06F-49C2-A10F-75ED3D06E647}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5133EA76-8FE5-4FCA-88A5-022C89FBA9B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SXM" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
     <sheet name="Sheet2" sheetId="8" r:id="rId7"/>
     <sheet name="Sheet1" sheetId="7" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="191029" calcCompleted="0"/>
+  <calcPr calcId="191029" iterateCount="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="62">
   <si>
     <t>SXM</t>
   </si>
@@ -276,6 +276,9 @@
   </si>
   <si>
     <t>Values</t>
+  </si>
+  <si>
+    <t>Medium</t>
   </si>
 </sst>
 </file>
@@ -10164,16 +10167,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="F18:F20"/>
+    <mergeCell ref="D18:D20"/>
+    <mergeCell ref="H4:H6"/>
+    <mergeCell ref="H11:H13"/>
+    <mergeCell ref="H18:H20"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="D4:D6"/>
     <mergeCell ref="F4:F6"/>
     <mergeCell ref="D11:D13"/>
     <mergeCell ref="F11:F13"/>
-    <mergeCell ref="F18:F20"/>
-    <mergeCell ref="D18:D20"/>
-    <mergeCell ref="H4:H6"/>
-    <mergeCell ref="H11:H13"/>
-    <mergeCell ref="H18:H20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -10183,10 +10186,10 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7C6C772-549F-407B-A6B9-32F2ED2FF002}">
-  <dimension ref="B1:J13"/>
+  <dimension ref="B1:J37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="2:10" ht="15" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
@@ -10199,6 +10202,9 @@
       <c r="E1" s="3" t="s">
         <v>56</v>
       </c>
+      <c r="H1" s="3" t="s">
+        <v>61</v>
+      </c>
       <c r="I1" t="s">
         <v>59</v>
       </c>
@@ -10219,10 +10225,13 @@
       <c r="E2" s="30">
         <v>0.907796706908784</v>
       </c>
+      <c r="H2" t="s">
+        <v>0</v>
+      </c>
       <c r="I2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="29">
+      <c r="J2" s="18">
         <v>1</v>
       </c>
     </row>
@@ -10239,10 +10248,13 @@
       <c r="E3" s="30">
         <v>0.72588094045230001</v>
       </c>
+      <c r="H3" t="s">
+        <v>0</v>
+      </c>
       <c r="I3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J3" s="29">
+      <c r="J3" s="18">
         <v>1</v>
       </c>
     </row>
@@ -10259,82 +10271,376 @@
       <c r="E4" s="30">
         <v>1.09552739043026</v>
       </c>
+      <c r="H4" t="s">
+        <v>0</v>
+      </c>
       <c r="I4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="29">
+      <c r="J4" s="18">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="H5" t="s">
+        <v>0</v>
+      </c>
       <c r="I5" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="J5" s="30">
-        <v>14.9733609152594</v>
+      <c r="J5" s="6">
+        <v>16.198602961602301</v>
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="H6" t="s">
+        <v>0</v>
+      </c>
       <c r="I6" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="J6" s="30">
-        <v>27.052593296637198</v>
+      <c r="J6" s="19">
+        <v>13.804274206794499</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="H7" t="s">
+        <v>0</v>
+      </c>
       <c r="I7" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="J7" s="30">
-        <v>14.9664573834732</v>
+      <c r="J7" s="19">
+        <v>10.1757874311372</v>
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="H8" t="s">
+        <v>0</v>
+      </c>
       <c r="I8" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="J8" s="30">
-        <v>5.9602162784990798</v>
+      <c r="J8" s="6">
+        <v>2.6853007827131101</v>
       </c>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="H9" t="s">
+        <v>0</v>
+      </c>
       <c r="I9" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="J9" s="30">
-        <v>5.4274596746618302</v>
+      <c r="J9" s="19">
+        <v>5.2847912419250296</v>
       </c>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="H10" t="s">
+        <v>0</v>
+      </c>
       <c r="I10" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="J10" s="30">
-        <v>6.6906997447058503</v>
+      <c r="J10" s="19">
+        <v>2.2949259580686898</v>
       </c>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="H11" t="s">
+        <v>0</v>
+      </c>
       <c r="I11" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="J11" s="30">
-        <v>0.907796706908784</v>
+      <c r="J11" s="6">
+        <v>0.768230073493543</v>
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="H12" t="s">
+        <v>0</v>
+      </c>
       <c r="I12" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="J12" s="30">
-        <v>0.72588094045230001</v>
+      <c r="J12" s="19">
+        <v>0.95345954179455605</v>
       </c>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="H13" t="s">
+        <v>0</v>
+      </c>
       <c r="I13" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="J13" s="30">
+      <c r="J13" s="19">
+        <v>0.49657078173872798</v>
+      </c>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="H14" t="s">
+        <v>1</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J14" s="18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="H15" t="s">
+        <v>1</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J15" s="18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="H16" t="s">
+        <v>1</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J16" s="18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="8:10" x14ac:dyDescent="0.3">
+      <c r="H17" t="s">
+        <v>1</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="J17" s="6">
+        <v>4.9050852792114696</v>
+      </c>
+    </row>
+    <row r="18" spans="8:10" x14ac:dyDescent="0.3">
+      <c r="H18" t="s">
+        <v>1</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="J18" s="6">
+        <v>3.27066381576154</v>
+      </c>
+    </row>
+    <row r="19" spans="8:10" x14ac:dyDescent="0.3">
+      <c r="H19" t="s">
+        <v>1</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="J19" s="6">
+        <v>3.0340180410320898</v>
+      </c>
+    </row>
+    <row r="20" spans="8:10" x14ac:dyDescent="0.3">
+      <c r="H20" t="s">
+        <v>1</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="J20" s="6">
+        <v>2.0399913580878599</v>
+      </c>
+    </row>
+    <row r="21" spans="8:10" x14ac:dyDescent="0.3">
+      <c r="H21" t="s">
+        <v>1</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="J21" s="6">
+        <v>2.3162714657693901</v>
+      </c>
+    </row>
+    <row r="22" spans="8:10" x14ac:dyDescent="0.3">
+      <c r="H22" t="s">
+        <v>1</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="J22" s="6">
+        <v>1.29075916796628</v>
+      </c>
+    </row>
+    <row r="23" spans="8:10" x14ac:dyDescent="0.3">
+      <c r="H23" t="s">
+        <v>1</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="J23" s="6">
+        <v>1.01582147398281</v>
+      </c>
+    </row>
+    <row r="24" spans="8:10" x14ac:dyDescent="0.3">
+      <c r="H24" t="s">
+        <v>1</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="J24" s="6">
+        <v>1.2010572282274701</v>
+      </c>
+    </row>
+    <row r="25" spans="8:10" x14ac:dyDescent="0.3">
+      <c r="H25" t="s">
+        <v>1</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="J25" s="6">
+        <v>0.85764657453567605</v>
+      </c>
+    </row>
+    <row r="26" spans="8:10" x14ac:dyDescent="0.3">
+      <c r="H26" t="s">
+        <v>2</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J26" s="18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="8:10" x14ac:dyDescent="0.3">
+      <c r="H27" t="s">
+        <v>2</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J27" s="18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="8:10" x14ac:dyDescent="0.3">
+      <c r="H28" t="s">
+        <v>2</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J28" s="18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="8:10" x14ac:dyDescent="0.3">
+      <c r="H29" t="s">
+        <v>2</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="J29" s="6">
+        <v>14.9733609152594</v>
+      </c>
+    </row>
+    <row r="30" spans="8:10" x14ac:dyDescent="0.3">
+      <c r="H30" t="s">
+        <v>2</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="J30" s="6">
+        <v>27.052593296637198</v>
+      </c>
+    </row>
+    <row r="31" spans="8:10" x14ac:dyDescent="0.3">
+      <c r="H31" t="s">
+        <v>2</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="J31" s="6">
+        <v>14.9664573834732</v>
+      </c>
+    </row>
+    <row r="32" spans="8:10" x14ac:dyDescent="0.3">
+      <c r="H32" t="s">
+        <v>2</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="J32" s="6">
+        <v>5.9602162784990798</v>
+      </c>
+    </row>
+    <row r="33" spans="8:10" x14ac:dyDescent="0.3">
+      <c r="H33" t="s">
+        <v>2</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="J33" s="6">
+        <v>5.4274596746618302</v>
+      </c>
+    </row>
+    <row r="34" spans="8:10" x14ac:dyDescent="0.3">
+      <c r="H34" t="s">
+        <v>2</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="J34" s="6">
+        <v>6.6906997447058503</v>
+      </c>
+    </row>
+    <row r="35" spans="8:10" x14ac:dyDescent="0.3">
+      <c r="H35" t="s">
+        <v>2</v>
+      </c>
+      <c r="I35" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="J35" s="6">
+        <v>0.907796706908784</v>
+      </c>
+    </row>
+    <row r="36" spans="8:10" x14ac:dyDescent="0.3">
+      <c r="H36" t="s">
+        <v>2</v>
+      </c>
+      <c r="I36" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="J36" s="6">
+        <v>0.72588094045230001</v>
+      </c>
+    </row>
+    <row r="37" spans="8:10" x14ac:dyDescent="0.3">
+      <c r="H37" t="s">
+        <v>2</v>
+      </c>
+      <c r="I37" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="J37" s="6">
         <v>1.09552739043026</v>
       </c>
     </row>

</xml_diff>